<commit_message>
reduced requirements and docker dependency; removed themes; german is localization base
</commit_message>
<xml_diff>
--- a/import/locations.xlsx
+++ b/import/locations.xlsx
@@ -4691,10 +4691,10 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>50.5898433</v>
+        <v>50.590044</v>
       </c>
       <c r="G78" t="n">
-        <v>8.6780645</v>
+        <v>8.6786622</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>

</xml_diff>